<commit_message>
Update evaluation tables: AudioSeal and Timbre columns now populated
Snapshot at 2026-09-15 00:34. RT-SW detection and all five methods'
imperceptibility are complete; AudioSeal (150-250 clips), WavMark (200) and
Timbre (400) are partial, and SilentCipher has not yet checkpointed.

The phone-call row is the one to watch as N grows. RT-SW holds 0.900 accuracy
at AUC 0.956 where AudioSeal collapses to 0.531/0.563 and WavMark to
0.500/0.500 -- the latter being total sync failure, not chance-level accuracy,
since every positive scores exactly 8/16 like the negatives. Timbre sits in
between at 0.781/0.904.

The reverse holds under Gaussian noise, where RT-SW is weakest at 0.609/0.681
against Timbre 0.890/0.965 and AudioSeal 0.795/0.951.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/watermarking_model/results/evals/detection_metrics.xlsx
+++ b/watermarking_model/results/evals/detection_metrics.xlsx
@@ -1259,7 +1259,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="C18" t="n">
         <v>1</v>
@@ -1289,19 +1289,19 @@
         <v>1</v>
       </c>
       <c r="L18" t="n">
-        <v>0.981155</v>
+        <v>0.993638</v>
       </c>
       <c r="M18" t="n">
         <v>1</v>
       </c>
       <c r="N18" t="n">
-        <v>0.003333</v>
+        <v>0.007889</v>
       </c>
       <c r="O18" t="n">
-        <v>0.000883</v>
+        <v>0.003565</v>
       </c>
       <c r="P18" t="n">
-        <v>0.027774</v>
+        <v>0.019358</v>
       </c>
       <c r="Q18" t="n">
         <v>13</v>
@@ -1310,7 +1310,7 @@
         <v>1</v>
       </c>
       <c r="S18" t="n">
-        <v>0.00614</v>
+        <v>0.008389000000000001</v>
       </c>
     </row>
     <row r="19">
@@ -1320,7 +1320,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="C19" t="n">
         <v>1</v>
@@ -1350,19 +1350,19 @@
         <v>1</v>
       </c>
       <c r="L19" t="n">
-        <v>0.981155</v>
+        <v>0.993638</v>
       </c>
       <c r="M19" t="n">
         <v>1</v>
       </c>
       <c r="N19" t="n">
-        <v>0.006667</v>
+        <v>0.010778</v>
       </c>
       <c r="O19" t="n">
-        <v>0.000883</v>
+        <v>0.004591</v>
       </c>
       <c r="P19" t="n">
-        <v>0.027774</v>
+        <v>0.021644</v>
       </c>
       <c r="Q19" t="n">
         <v>13</v>
@@ -1371,7 +1371,7 @@
         <v>1</v>
       </c>
       <c r="S19" t="n">
-        <v>0.007368</v>
+        <v>0.011152</v>
       </c>
     </row>
     <row r="20">
@@ -1381,58 +1381,58 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="C20" t="n">
-        <v>0.799167</v>
+        <v>0.795042</v>
       </c>
       <c r="D20" t="n">
-        <v>0.122948</v>
+        <v>0.123665</v>
       </c>
       <c r="E20" t="n">
-        <v>0.008694</v>
+        <v>0.005049</v>
       </c>
       <c r="F20" t="n">
-        <v>0.772961</v>
+        <v>0.780522</v>
       </c>
       <c r="G20" t="n">
-        <v>0.807039</v>
+        <v>0.800312</v>
       </c>
       <c r="H20" t="n">
-        <v>0.96905</v>
+        <v>0.951219</v>
       </c>
       <c r="I20" t="n">
-        <v>0.946448</v>
+        <v>0.9371660000000001</v>
       </c>
       <c r="J20" t="n">
-        <v>0.9774659999999999</v>
+        <v>0.9592889999999999</v>
       </c>
       <c r="K20" t="n">
-        <v>0.573333</v>
+        <v>0.590333</v>
       </c>
       <c r="L20" t="n">
-        <v>0.470823</v>
+        <v>0.533415</v>
       </c>
       <c r="M20" t="n">
-        <v>0.607669</v>
+        <v>0.612318</v>
       </c>
       <c r="N20" t="n">
-        <v>0.006667</v>
+        <v>0.013222</v>
       </c>
       <c r="O20" t="n">
-        <v>0.000883</v>
+        <v>0.005663</v>
       </c>
       <c r="P20" t="n">
-        <v>0.027774</v>
+        <v>0.023884</v>
       </c>
       <c r="Q20" t="n">
         <v>13</v>
       </c>
       <c r="R20" t="n">
-        <v>0.61193</v>
+        <v>0.594216</v>
       </c>
       <c r="S20" t="n">
-        <v>0.010877</v>
+        <v>0.014061</v>
       </c>
     </row>
     <row r="21">
@@ -1442,7 +1442,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="C21" t="n">
         <v>1</v>
@@ -1472,19 +1472,19 @@
         <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>0.981155</v>
+        <v>0.993638</v>
       </c>
       <c r="M21" t="n">
         <v>1</v>
       </c>
       <c r="N21" t="n">
-        <v>0.003333</v>
+        <v>0.009556</v>
       </c>
       <c r="O21" t="n">
-        <v>0.000883</v>
+        <v>0.004591</v>
       </c>
       <c r="P21" t="n">
-        <v>0.027774</v>
+        <v>0.021644</v>
       </c>
       <c r="Q21" t="n">
         <v>13</v>
@@ -1493,7 +1493,7 @@
         <v>1</v>
       </c>
       <c r="S21" t="n">
-        <v>0.008947</v>
+        <v>0.010109</v>
       </c>
     </row>
     <row r="22">
@@ -1503,7 +1503,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="C22" t="n">
         <v>1</v>
@@ -1533,19 +1533,19 @@
         <v>1</v>
       </c>
       <c r="L22" t="n">
-        <v>0.981155</v>
+        <v>0.993638</v>
       </c>
       <c r="M22" t="n">
         <v>1</v>
       </c>
       <c r="N22" t="n">
-        <v>0.006667</v>
+        <v>0.009889</v>
       </c>
       <c r="O22" t="n">
-        <v>0.000883</v>
+        <v>0.004591</v>
       </c>
       <c r="P22" t="n">
-        <v>0.027774</v>
+        <v>0.021644</v>
       </c>
       <c r="Q22" t="n">
         <v>13</v>
@@ -1554,7 +1554,7 @@
         <v>1</v>
       </c>
       <c r="S22" t="n">
-        <v>0.010175</v>
+        <v>0.010616</v>
       </c>
     </row>
     <row r="23">
@@ -1564,7 +1564,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="C23" t="n">
         <v>1</v>
@@ -1594,19 +1594,19 @@
         <v>1</v>
       </c>
       <c r="L23" t="n">
-        <v>0.981155</v>
+        <v>0.993638</v>
       </c>
       <c r="M23" t="n">
         <v>1</v>
       </c>
       <c r="N23" t="n">
-        <v>0</v>
+        <v>0.007111</v>
       </c>
       <c r="O23" t="n">
-        <v>0</v>
+        <v>0.002596</v>
       </c>
       <c r="P23" t="n">
-        <v>0.018845</v>
+        <v>0.017015</v>
       </c>
       <c r="Q23" t="n">
         <v>13</v>
@@ -1615,7 +1615,7 @@
         <v>1</v>
       </c>
       <c r="S23" t="n">
-        <v>0.001404</v>
+        <v>0.007611</v>
       </c>
     </row>
     <row r="24">
@@ -1625,7 +1625,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="C24" t="n">
         <v>1</v>
@@ -1655,19 +1655,19 @@
         <v>1</v>
       </c>
       <c r="L24" t="n">
-        <v>0.981155</v>
+        <v>0.993638</v>
       </c>
       <c r="M24" t="n">
         <v>1</v>
       </c>
       <c r="N24" t="n">
-        <v>0.003333</v>
+        <v>0.007889</v>
       </c>
       <c r="O24" t="n">
-        <v>0.000883</v>
+        <v>0.003565</v>
       </c>
       <c r="P24" t="n">
-        <v>0.027774</v>
+        <v>0.019358</v>
       </c>
       <c r="Q24" t="n">
         <v>13</v>
@@ -1676,7 +1676,7 @@
         <v>1</v>
       </c>
       <c r="S24" t="n">
-        <v>0.00614</v>
+        <v>0.008389000000000001</v>
       </c>
     </row>
     <row r="25">
@@ -1686,7 +1686,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="C25" t="n">
         <v>1</v>
@@ -1716,19 +1716,19 @@
         <v>1</v>
       </c>
       <c r="L25" t="n">
-        <v>0.981155</v>
+        <v>0.993638</v>
       </c>
       <c r="M25" t="n">
         <v>1</v>
       </c>
       <c r="N25" t="n">
-        <v>0.01</v>
+        <v>0.013111</v>
       </c>
       <c r="O25" t="n">
-        <v>0.002747</v>
+        <v>0.006771</v>
       </c>
       <c r="P25" t="n">
-        <v>0.035722</v>
+        <v>0.026087</v>
       </c>
       <c r="Q25" t="n">
         <v>13</v>
@@ -1737,7 +1737,7 @@
         <v>1</v>
       </c>
       <c r="S25" t="n">
-        <v>0.012807</v>
+        <v>0.013888</v>
       </c>
     </row>
     <row r="26">
@@ -1747,58 +1747,58 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="C26" t="n">
-        <v>0.996458</v>
+        <v>0.99825</v>
       </c>
       <c r="D26" t="n">
-        <v>0.031795</v>
+        <v>0.019216</v>
       </c>
       <c r="E26" t="n">
-        <v>0.002248</v>
+        <v>0.000785</v>
       </c>
       <c r="F26" t="n">
-        <v>0.992469</v>
+        <v>0.9969</v>
       </c>
       <c r="G26" t="n">
-        <v>1.001281</v>
+        <v>0.9999749999999999</v>
       </c>
       <c r="H26" t="n">
-        <v>0.9982</v>
+        <v>0.999281</v>
       </c>
       <c r="I26" t="n">
-        <v>0.995762</v>
+        <v>0.998354</v>
       </c>
       <c r="J26" t="n">
         <v>1</v>
       </c>
       <c r="K26" t="n">
-        <v>0.993333</v>
+        <v>0.9977780000000001</v>
       </c>
       <c r="L26" t="n">
-        <v>0.972226</v>
+        <v>0.9906199999999999</v>
       </c>
       <c r="M26" t="n">
-        <v>0.999117</v>
+        <v>0.999706</v>
       </c>
       <c r="N26" t="n">
-        <v>0.006667</v>
+        <v>0.010111</v>
       </c>
       <c r="O26" t="n">
-        <v>0.002747</v>
+        <v>0.004591</v>
       </c>
       <c r="P26" t="n">
-        <v>0.035722</v>
+        <v>0.021644</v>
       </c>
       <c r="Q26" t="n">
         <v>13</v>
       </c>
       <c r="R26" t="n">
-        <v>0.993333</v>
+        <v>0.9977780000000001</v>
       </c>
       <c r="S26" t="n">
-        <v>0.015789</v>
+        <v>0.011115</v>
       </c>
     </row>
     <row r="27">
@@ -1808,58 +1808,58 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="C27" t="n">
-        <v>0.555</v>
+        <v>0.530896</v>
       </c>
       <c r="D27" t="n">
-        <v>0.131937</v>
+        <v>0.125151</v>
       </c>
       <c r="E27" t="n">
-        <v>0.009329</v>
+        <v>0.005109</v>
       </c>
       <c r="F27" t="n">
-        <v>0.535152</v>
+        <v>0.5200900000000001</v>
       </c>
       <c r="G27" t="n">
-        <v>0.571723</v>
+        <v>0.540118</v>
       </c>
       <c r="H27" t="n">
-        <v>0.612567</v>
+        <v>0.5629459999999999</v>
       </c>
       <c r="I27" t="n">
-        <v>0.555246</v>
+        <v>0.527917</v>
       </c>
       <c r="J27" t="n">
-        <v>0.666431</v>
+        <v>0.593959</v>
       </c>
       <c r="K27" t="n">
-        <v>0.036667</v>
+        <v>0.018889</v>
       </c>
       <c r="L27" t="n">
-        <v>0.017056</v>
+        <v>0.011477</v>
       </c>
       <c r="M27" t="n">
-        <v>0.07047100000000001</v>
+        <v>0.03463</v>
       </c>
       <c r="N27" t="n">
-        <v>0.013333</v>
+        <v>0.006111</v>
       </c>
       <c r="O27" t="n">
-        <v>0.002747</v>
+        <v>0.001702</v>
       </c>
       <c r="P27" t="n">
-        <v>0.035722</v>
+        <v>0.014596</v>
       </c>
       <c r="Q27" t="n">
         <v>13</v>
       </c>
       <c r="R27" t="n">
-        <v>0.054912</v>
+        <v>0.0202</v>
       </c>
       <c r="S27" t="n">
-        <v>0.016842</v>
+        <v>0.006894</v>
       </c>
     </row>
     <row r="29">
@@ -4136,7 +4136,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="C18" t="n">
         <v>1</v>
@@ -4166,19 +4166,19 @@
         <v>1</v>
       </c>
       <c r="L18" t="n">
-        <v>0.928652</v>
+        <v>0.97503</v>
       </c>
       <c r="M18" t="n">
         <v>1</v>
       </c>
       <c r="N18" t="n">
-        <v>0</v>
+        <v>0.006667</v>
       </c>
       <c r="O18" t="n">
-        <v>0</v>
+        <v>0.001178</v>
       </c>
       <c r="P18" t="n">
-        <v>0.07134799999999999</v>
+        <v>0.036793</v>
       </c>
       <c r="Q18" t="n">
         <v>13</v>
@@ -4187,7 +4187,7 @@
         <v>1</v>
       </c>
       <c r="S18" t="n">
-        <v>0</v>
+        <v>0.006834</v>
       </c>
     </row>
     <row r="19">
@@ -4197,7 +4197,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="C19" t="n">
         <v>1</v>
@@ -4227,19 +4227,19 @@
         <v>1</v>
       </c>
       <c r="L19" t="n">
-        <v>0.928652</v>
+        <v>0.97503</v>
       </c>
       <c r="M19" t="n">
         <v>1</v>
       </c>
       <c r="N19" t="n">
-        <v>0</v>
+        <v>0.013333</v>
       </c>
       <c r="O19" t="n">
-        <v>0</v>
+        <v>0.003664</v>
       </c>
       <c r="P19" t="n">
-        <v>0.07134799999999999</v>
+        <v>0.047307</v>
       </c>
       <c r="Q19" t="n">
         <v>13</v>
@@ -4248,7 +4248,7 @@
         <v>1</v>
       </c>
       <c r="S19" t="n">
-        <v>0</v>
+        <v>0.013501</v>
       </c>
     </row>
     <row r="20">
@@ -4258,58 +4258,58 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="C20" t="n">
         <v>0.8125</v>
       </c>
       <c r="D20" t="n">
-        <v>0.123718</v>
+        <v>0.123311</v>
       </c>
       <c r="E20" t="n">
-        <v>0.017496</v>
+        <v>0.010068</v>
       </c>
       <c r="F20" t="n">
-        <v>0.778208</v>
+        <v>0.792767</v>
       </c>
       <c r="G20" t="n">
-        <v>0.846792</v>
+        <v>0.832233</v>
       </c>
       <c r="H20" t="n">
-        <v>0.9698</v>
+        <v>0.945444</v>
       </c>
       <c r="I20" t="n">
-        <v>0.935995</v>
+        <v>0.918303</v>
       </c>
       <c r="J20" t="n">
-        <v>0.9936</v>
+        <v>0.968297</v>
       </c>
       <c r="K20" t="n">
-        <v>0.62</v>
+        <v>0.66</v>
       </c>
       <c r="L20" t="n">
-        <v>0.481504</v>
+        <v>0.581043</v>
       </c>
       <c r="M20" t="n">
-        <v>0.741372</v>
+        <v>0.730967</v>
       </c>
       <c r="N20" t="n">
-        <v>0.02</v>
+        <v>0.026667</v>
       </c>
       <c r="O20" t="n">
-        <v>0.003539</v>
+        <v>0.010418</v>
       </c>
       <c r="P20" t="n">
-        <v>0.104954</v>
+        <v>0.066554</v>
       </c>
       <c r="Q20" t="n">
         <v>13</v>
       </c>
       <c r="R20" t="n">
-        <v>0.653684</v>
+        <v>0.663019</v>
       </c>
       <c r="S20" t="n">
-        <v>0.024211</v>
+        <v>0.028176</v>
       </c>
     </row>
     <row r="21">
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="C21" t="n">
         <v>1</v>
@@ -4349,19 +4349,19 @@
         <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>0.928652</v>
+        <v>0.97503</v>
       </c>
       <c r="M21" t="n">
         <v>1</v>
       </c>
       <c r="N21" t="n">
-        <v>0</v>
+        <v>0.006667</v>
       </c>
       <c r="O21" t="n">
-        <v>0</v>
+        <v>0.001178</v>
       </c>
       <c r="P21" t="n">
-        <v>0.07134799999999999</v>
+        <v>0.036793</v>
       </c>
       <c r="Q21" t="n">
         <v>13</v>
@@ -4370,7 +4370,7 @@
         <v>1</v>
       </c>
       <c r="S21" t="n">
-        <v>0</v>
+        <v>0.00717</v>
       </c>
     </row>
     <row r="22">
@@ -4380,7 +4380,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="C22" t="n">
         <v>1</v>
@@ -4410,19 +4410,19 @@
         <v>1</v>
       </c>
       <c r="L22" t="n">
-        <v>0.928652</v>
+        <v>0.97503</v>
       </c>
       <c r="M22" t="n">
         <v>1</v>
       </c>
       <c r="N22" t="n">
-        <v>0</v>
+        <v>0.006667</v>
       </c>
       <c r="O22" t="n">
-        <v>0</v>
+        <v>0.001178</v>
       </c>
       <c r="P22" t="n">
-        <v>0.07134799999999999</v>
+        <v>0.036793</v>
       </c>
       <c r="Q22" t="n">
         <v>13</v>
@@ -4431,7 +4431,7 @@
         <v>1</v>
       </c>
       <c r="S22" t="n">
-        <v>0</v>
+        <v>0.007338</v>
       </c>
     </row>
     <row r="23">
@@ -4441,7 +4441,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="C23" t="n">
         <v>1</v>
@@ -4471,19 +4471,19 @@
         <v>1</v>
       </c>
       <c r="L23" t="n">
-        <v>0.928652</v>
+        <v>0.97503</v>
       </c>
       <c r="M23" t="n">
         <v>1</v>
       </c>
       <c r="N23" t="n">
-        <v>0</v>
+        <v>0.013333</v>
       </c>
       <c r="O23" t="n">
-        <v>0</v>
+        <v>0.003664</v>
       </c>
       <c r="P23" t="n">
-        <v>0.07134799999999999</v>
+        <v>0.047307</v>
       </c>
       <c r="Q23" t="n">
         <v>13</v>
@@ -4492,7 +4492,7 @@
         <v>1</v>
       </c>
       <c r="S23" t="n">
-        <v>0</v>
+        <v>0.013501</v>
       </c>
     </row>
     <row r="24">
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="C24" t="n">
         <v>1</v>
@@ -4532,19 +4532,19 @@
         <v>1</v>
       </c>
       <c r="L24" t="n">
-        <v>0.928652</v>
+        <v>0.97503</v>
       </c>
       <c r="M24" t="n">
         <v>1</v>
       </c>
       <c r="N24" t="n">
-        <v>0</v>
+        <v>0.006667</v>
       </c>
       <c r="O24" t="n">
-        <v>0</v>
+        <v>0.001178</v>
       </c>
       <c r="P24" t="n">
-        <v>0.07134799999999999</v>
+        <v>0.036793</v>
       </c>
       <c r="Q24" t="n">
         <v>13</v>
@@ -4553,7 +4553,7 @@
         <v>1</v>
       </c>
       <c r="S24" t="n">
-        <v>0</v>
+        <v>0.006834</v>
       </c>
     </row>
     <row r="25">
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="C25" t="n">
         <v>1</v>
@@ -4593,19 +4593,19 @@
         <v>1</v>
       </c>
       <c r="L25" t="n">
-        <v>0.928652</v>
+        <v>0.97503</v>
       </c>
       <c r="M25" t="n">
         <v>1</v>
       </c>
       <c r="N25" t="n">
-        <v>0</v>
+        <v>0.013333</v>
       </c>
       <c r="O25" t="n">
-        <v>0</v>
+        <v>0.003664</v>
       </c>
       <c r="P25" t="n">
-        <v>0.07134799999999999</v>
+        <v>0.047307</v>
       </c>
       <c r="Q25" t="n">
         <v>13</v>
@@ -4614,7 +4614,7 @@
         <v>1</v>
       </c>
       <c r="S25" t="n">
-        <v>0</v>
+        <v>0.014004</v>
       </c>
     </row>
     <row r="26">
@@ -4624,58 +4624,58 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="C26" t="n">
-        <v>0.99125</v>
+        <v>0.99625</v>
       </c>
       <c r="D26" t="n">
-        <v>0.061872</v>
+        <v>0.036371</v>
       </c>
       <c r="E26" t="n">
-        <v>0.008750000000000001</v>
+        <v>0.00297</v>
       </c>
       <c r="F26" t="n">
-        <v>0.9741</v>
+        <v>0.990429</v>
       </c>
       <c r="G26" t="n">
-        <v>1.0084</v>
+        <v>1.002071</v>
       </c>
       <c r="H26" t="n">
-        <v>0.9946</v>
+        <v>0.997844</v>
       </c>
       <c r="I26" t="n">
-        <v>0.982</v>
+        <v>0.992667</v>
       </c>
       <c r="J26" t="n">
         <v>1</v>
       </c>
       <c r="K26" t="n">
-        <v>0.98</v>
+        <v>0.993333</v>
       </c>
       <c r="L26" t="n">
-        <v>0.895046</v>
+        <v>0.963207</v>
       </c>
       <c r="M26" t="n">
-        <v>0.996461</v>
+        <v>0.998822</v>
       </c>
       <c r="N26" t="n">
-        <v>0</v>
+        <v>0.013333</v>
       </c>
       <c r="O26" t="n">
-        <v>0</v>
+        <v>0.003664</v>
       </c>
       <c r="P26" t="n">
-        <v>0.07134799999999999</v>
+        <v>0.047307</v>
       </c>
       <c r="Q26" t="n">
         <v>13</v>
       </c>
       <c r="R26" t="n">
-        <v>0.98</v>
+        <v>0.993333</v>
       </c>
       <c r="S26" t="n">
-        <v>0.008421</v>
+        <v>0.014004</v>
       </c>
     </row>
     <row r="27">
@@ -4685,58 +4685,58 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="C27" t="n">
-        <v>0.54875</v>
+        <v>0.5325</v>
       </c>
       <c r="D27" t="n">
-        <v>0.128949</v>
+        <v>0.118479</v>
       </c>
       <c r="E27" t="n">
-        <v>0.018236</v>
+        <v>0.009674</v>
       </c>
       <c r="F27" t="n">
-        <v>0.513008</v>
+        <v>0.51354</v>
       </c>
       <c r="G27" t="n">
-        <v>0.584492</v>
+        <v>0.55146</v>
       </c>
       <c r="H27" t="n">
-        <v>0.6112</v>
+        <v>0.579956</v>
       </c>
       <c r="I27" t="n">
-        <v>0.498575</v>
+        <v>0.513798</v>
       </c>
       <c r="J27" t="n">
-        <v>0.72201</v>
+        <v>0.6444260000000001</v>
       </c>
       <c r="K27" t="n">
-        <v>0.02</v>
+        <v>0.006667</v>
       </c>
       <c r="L27" t="n">
-        <v>0.003539</v>
+        <v>0.001178</v>
       </c>
       <c r="M27" t="n">
-        <v>0.104954</v>
+        <v>0.036793</v>
       </c>
       <c r="N27" t="n">
-        <v>0.02</v>
+        <v>0.013333</v>
       </c>
       <c r="O27" t="n">
-        <v>0.003539</v>
+        <v>0.003664</v>
       </c>
       <c r="P27" t="n">
-        <v>0.104954</v>
+        <v>0.047307</v>
       </c>
       <c r="Q27" t="n">
         <v>13</v>
       </c>
       <c r="R27" t="n">
-        <v>0.045263</v>
+        <v>0.008512</v>
       </c>
       <c r="S27" t="n">
-        <v>0.02</v>
+        <v>0.014172</v>
       </c>
     </row>
     <row r="29">
@@ -7013,7 +7013,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="C18" t="n">
         <v>1</v>
@@ -7043,19 +7043,19 @@
         <v>1</v>
       </c>
       <c r="L18" t="n">
-        <v>0.928652</v>
+        <v>0.981155</v>
       </c>
       <c r="M18" t="n">
         <v>1</v>
       </c>
       <c r="N18" t="n">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="O18" t="n">
-        <v>0</v>
+        <v>0.000883</v>
       </c>
       <c r="P18" t="n">
-        <v>0.07134799999999999</v>
+        <v>0.027774</v>
       </c>
       <c r="Q18" t="n">
         <v>13</v>
@@ -7064,7 +7064,7 @@
         <v>1</v>
       </c>
       <c r="S18" t="n">
-        <v>0.004211</v>
+        <v>0.005629</v>
       </c>
     </row>
     <row r="19">
@@ -7074,7 +7074,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="C19" t="n">
         <v>1</v>
@@ -7104,19 +7104,19 @@
         <v>1</v>
       </c>
       <c r="L19" t="n">
-        <v>0.928652</v>
+        <v>0.981155</v>
       </c>
       <c r="M19" t="n">
         <v>1</v>
       </c>
       <c r="N19" t="n">
-        <v>0.02</v>
+        <v>0.015</v>
       </c>
       <c r="O19" t="n">
-        <v>0.003539</v>
+        <v>0.005114</v>
       </c>
       <c r="P19" t="n">
-        <v>0.104954</v>
+        <v>0.043166</v>
       </c>
       <c r="Q19" t="n">
         <v>13</v>
@@ -7125,7 +7125,7 @@
         <v>1</v>
       </c>
       <c r="S19" t="n">
-        <v>0.02</v>
+        <v>0.015252</v>
       </c>
     </row>
     <row r="20">
@@ -7135,58 +7135,58 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="C20" t="n">
-        <v>0.8225</v>
+        <v>0.815625</v>
       </c>
       <c r="D20" t="n">
-        <v>0.093097</v>
+        <v>0.102717</v>
       </c>
       <c r="E20" t="n">
-        <v>0.013166</v>
+        <v>0.007263</v>
       </c>
       <c r="F20" t="n">
-        <v>0.796695</v>
+        <v>0.801389</v>
       </c>
       <c r="G20" t="n">
-        <v>0.848305</v>
+        <v>0.829861</v>
       </c>
       <c r="H20" t="n">
-        <v>0.9893999999999999</v>
+        <v>0.9779870000000001</v>
       </c>
       <c r="I20" t="n">
-        <v>0.9746</v>
+        <v>0.9665820000000001</v>
       </c>
       <c r="J20" t="n">
-        <v>0.9986</v>
+        <v>0.987726</v>
       </c>
       <c r="K20" t="n">
-        <v>0.66</v>
+        <v>0.655</v>
       </c>
       <c r="L20" t="n">
-        <v>0.5215379999999999</v>
+        <v>0.5867560000000001</v>
       </c>
       <c r="M20" t="n">
-        <v>0.775631</v>
+        <v>0.717402</v>
       </c>
       <c r="N20" t="n">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="O20" t="n">
-        <v>0</v>
+        <v>0.000883</v>
       </c>
       <c r="P20" t="n">
-        <v>0.07134799999999999</v>
+        <v>0.027774</v>
       </c>
       <c r="Q20" t="n">
         <v>13</v>
       </c>
       <c r="R20" t="n">
-        <v>0.7063160000000001</v>
+        <v>0.659403</v>
       </c>
       <c r="S20" t="n">
-        <v>0.004211</v>
+        <v>0.005503</v>
       </c>
     </row>
     <row r="21">
@@ -7196,7 +7196,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="C21" t="n">
         <v>1</v>
@@ -7226,19 +7226,19 @@
         <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>0.928652</v>
+        <v>0.981155</v>
       </c>
       <c r="M21" t="n">
         <v>1</v>
       </c>
       <c r="N21" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="O21" t="n">
-        <v>0</v>
+        <v>0.002747</v>
       </c>
       <c r="P21" t="n">
-        <v>0.07134799999999999</v>
+        <v>0.035722</v>
       </c>
       <c r="Q21" t="n">
         <v>13</v>
@@ -7247,7 +7247,7 @@
         <v>1</v>
       </c>
       <c r="S21" t="n">
-        <v>0.012632</v>
+        <v>0.010755</v>
       </c>
     </row>
     <row r="22">
@@ -7257,7 +7257,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="C22" t="n">
         <v>1</v>
@@ -7287,19 +7287,19 @@
         <v>1</v>
       </c>
       <c r="L22" t="n">
-        <v>0.928652</v>
+        <v>0.981155</v>
       </c>
       <c r="M22" t="n">
         <v>1</v>
       </c>
       <c r="N22" t="n">
-        <v>0.02</v>
+        <v>0.015</v>
       </c>
       <c r="O22" t="n">
-        <v>0.003539</v>
+        <v>0.005114</v>
       </c>
       <c r="P22" t="n">
-        <v>0.104954</v>
+        <v>0.043166</v>
       </c>
       <c r="Q22" t="n">
         <v>13</v>
@@ -7308,7 +7308,7 @@
         <v>1</v>
       </c>
       <c r="S22" t="n">
-        <v>0.024211</v>
+        <v>0.015503</v>
       </c>
     </row>
     <row r="23">
@@ -7318,7 +7318,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="C23" t="n">
         <v>1</v>
@@ -7348,7 +7348,7 @@
         <v>1</v>
       </c>
       <c r="L23" t="n">
-        <v>0.928652</v>
+        <v>0.981155</v>
       </c>
       <c r="M23" t="n">
         <v>1</v>
@@ -7360,7 +7360,7 @@
         <v>0</v>
       </c>
       <c r="P23" t="n">
-        <v>0.07134799999999999</v>
+        <v>0.018845</v>
       </c>
       <c r="Q23" t="n">
         <v>13</v>
@@ -7369,7 +7369,7 @@
         <v>1</v>
       </c>
       <c r="S23" t="n">
-        <v>0</v>
+        <v>0.000629</v>
       </c>
     </row>
     <row r="24">
@@ -7379,7 +7379,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="C24" t="n">
         <v>1</v>
@@ -7409,19 +7409,19 @@
         <v>1</v>
       </c>
       <c r="L24" t="n">
-        <v>0.928652</v>
+        <v>0.981155</v>
       </c>
       <c r="M24" t="n">
         <v>1</v>
       </c>
       <c r="N24" t="n">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="O24" t="n">
-        <v>0</v>
+        <v>0.000883</v>
       </c>
       <c r="P24" t="n">
-        <v>0.07134799999999999</v>
+        <v>0.027774</v>
       </c>
       <c r="Q24" t="n">
         <v>13</v>
@@ -7430,7 +7430,7 @@
         <v>1</v>
       </c>
       <c r="S24" t="n">
-        <v>0.004211</v>
+        <v>0.005629</v>
       </c>
     </row>
     <row r="25">
@@ -7440,7 +7440,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="C25" t="n">
         <v>1</v>
@@ -7470,19 +7470,19 @@
         <v>1</v>
       </c>
       <c r="L25" t="n">
-        <v>0.928652</v>
+        <v>0.981155</v>
       </c>
       <c r="M25" t="n">
         <v>1</v>
       </c>
       <c r="N25" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="O25" t="n">
-        <v>0.003539</v>
+        <v>0.002747</v>
       </c>
       <c r="P25" t="n">
-        <v>0.104954</v>
+        <v>0.035722</v>
       </c>
       <c r="Q25" t="n">
         <v>13</v>
@@ -7491,7 +7491,7 @@
         <v>1</v>
       </c>
       <c r="S25" t="n">
-        <v>0.02</v>
+        <v>0.010755</v>
       </c>
     </row>
     <row r="26">
@@ -7501,7 +7501,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="C26" t="n">
         <v>1</v>
@@ -7531,19 +7531,19 @@
         <v>1</v>
       </c>
       <c r="L26" t="n">
-        <v>0.928652</v>
+        <v>0.981155</v>
       </c>
       <c r="M26" t="n">
         <v>1</v>
       </c>
       <c r="N26" t="n">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="O26" t="n">
-        <v>0</v>
+        <v>0.000883</v>
       </c>
       <c r="P26" t="n">
-        <v>0.07134799999999999</v>
+        <v>0.027774</v>
       </c>
       <c r="Q26" t="n">
         <v>13</v>
@@ -7552,7 +7552,7 @@
         <v>1</v>
       </c>
       <c r="S26" t="n">
-        <v>0.012632</v>
+        <v>0.006635</v>
       </c>
     </row>
     <row r="27">
@@ -7562,58 +7562,58 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="C27" t="n">
-        <v>0.5675</v>
+        <v>0.537188</v>
       </c>
       <c r="D27" t="n">
-        <v>0.133535</v>
+        <v>0.129033</v>
       </c>
       <c r="E27" t="n">
-        <v>0.018885</v>
+        <v>0.009124</v>
       </c>
       <c r="F27" t="n">
-        <v>0.530487</v>
+        <v>0.519305</v>
       </c>
       <c r="G27" t="n">
-        <v>0.604513</v>
+        <v>0.55507</v>
       </c>
       <c r="H27" t="n">
-        <v>0.6258</v>
+        <v>0.56525</v>
       </c>
       <c r="I27" t="n">
-        <v>0.519755</v>
+        <v>0.51131</v>
       </c>
       <c r="J27" t="n">
-        <v>0.726805</v>
+        <v>0.620413</v>
       </c>
       <c r="K27" t="n">
-        <v>0.06</v>
+        <v>0.03</v>
       </c>
       <c r="L27" t="n">
-        <v>0.020615</v>
+        <v>0.01382</v>
       </c>
       <c r="M27" t="n">
-        <v>0.162171</v>
+        <v>0.06389400000000001</v>
       </c>
       <c r="N27" t="n">
-        <v>0.02</v>
+        <v>0.005</v>
       </c>
       <c r="O27" t="n">
-        <v>0.003539</v>
+        <v>0.000883</v>
       </c>
       <c r="P27" t="n">
-        <v>0.104954</v>
+        <v>0.027774</v>
       </c>
       <c r="Q27" t="n">
         <v>13</v>
       </c>
       <c r="R27" t="n">
-        <v>0.072632</v>
+        <v>0.030881</v>
       </c>
       <c r="S27" t="n">
-        <v>0.024211</v>
+        <v>0.006006</v>
       </c>
     </row>
     <row r="29">
@@ -9890,7 +9890,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="C18" t="n">
         <v>1</v>
@@ -9920,19 +9920,19 @@
         <v>1</v>
       </c>
       <c r="L18" t="n">
-        <v>0.9630069999999999</v>
+        <v>0.984867</v>
       </c>
       <c r="M18" t="n">
         <v>1</v>
       </c>
       <c r="N18" t="n">
-        <v>0.01</v>
+        <v>0.012</v>
       </c>
       <c r="O18" t="n">
-        <v>0.001767</v>
+        <v>0.004089</v>
       </c>
       <c r="P18" t="n">
-        <v>0.054486</v>
+        <v>0.034681</v>
       </c>
       <c r="Q18" t="n">
         <v>13</v>
@@ -9941,7 +9941,7 @@
         <v>1</v>
       </c>
       <c r="S18" t="n">
-        <v>0.014211</v>
+        <v>0.012704</v>
       </c>
     </row>
     <row r="19">
@@ -9951,7 +9951,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="C19" t="n">
         <v>1</v>
@@ -9981,19 +9981,19 @@
         <v>1</v>
       </c>
       <c r="L19" t="n">
-        <v>0.9630069999999999</v>
+        <v>0.984867</v>
       </c>
       <c r="M19" t="n">
         <v>1</v>
       </c>
       <c r="N19" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
       <c r="O19" t="n">
-        <v>0</v>
+        <v>0.000706</v>
       </c>
       <c r="P19" t="n">
-        <v>0.036993</v>
+        <v>0.022306</v>
       </c>
       <c r="Q19" t="n">
         <v>13</v>
@@ -10002,7 +10002,7 @@
         <v>1</v>
       </c>
       <c r="S19" t="n">
-        <v>0.002105</v>
+        <v>0.004704</v>
       </c>
     </row>
     <row r="20">
@@ -10012,58 +10012,58 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="C20" t="n">
-        <v>0.7625</v>
+        <v>0.757</v>
       </c>
       <c r="D20" t="n">
-        <v>0.130256</v>
+        <v>0.131654</v>
       </c>
       <c r="E20" t="n">
-        <v>0.013026</v>
+        <v>0.008326999999999999</v>
       </c>
       <c r="F20" t="n">
-        <v>0.73697</v>
+        <v>0.74068</v>
       </c>
       <c r="G20" t="n">
-        <v>0.78803</v>
+        <v>0.77332</v>
       </c>
       <c r="H20" t="n">
-        <v>0.94795</v>
+        <v>0.9302240000000001</v>
       </c>
       <c r="I20" t="n">
-        <v>0.92055</v>
+        <v>0.91047</v>
       </c>
       <c r="J20" t="n">
-        <v>0.9717</v>
+        <v>0.948041</v>
       </c>
       <c r="K20" t="n">
-        <v>0.44</v>
+        <v>0.456</v>
       </c>
       <c r="L20" t="n">
-        <v>0.34672</v>
+        <v>0.395392</v>
       </c>
       <c r="M20" t="n">
-        <v>0.5377189999999999</v>
+        <v>0.51794</v>
       </c>
       <c r="N20" t="n">
-        <v>0</v>
+        <v>0.008</v>
       </c>
       <c r="O20" t="n">
-        <v>0</v>
+        <v>0.002197</v>
       </c>
       <c r="P20" t="n">
-        <v>0.036993</v>
+        <v>0.028695</v>
       </c>
       <c r="Q20" t="n">
         <v>13</v>
       </c>
       <c r="R20" t="n">
-        <v>0.475789</v>
+        <v>0.460226</v>
       </c>
       <c r="S20" t="n">
-        <v>0.004211</v>
+        <v>0.008503</v>
       </c>
     </row>
     <row r="21">
@@ -10073,7 +10073,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="C21" t="n">
         <v>1</v>
@@ -10103,19 +10103,19 @@
         <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>0.9630069999999999</v>
+        <v>0.984867</v>
       </c>
       <c r="M21" t="n">
         <v>1</v>
       </c>
       <c r="N21" t="n">
-        <v>0.01</v>
+        <v>0.012</v>
       </c>
       <c r="O21" t="n">
-        <v>0.001767</v>
+        <v>0.004089</v>
       </c>
       <c r="P21" t="n">
-        <v>0.054486</v>
+        <v>0.034681</v>
       </c>
       <c r="Q21" t="n">
         <v>13</v>
@@ -10124,7 +10124,7 @@
         <v>1</v>
       </c>
       <c r="S21" t="n">
-        <v>0.014211</v>
+        <v>0.012403</v>
       </c>
     </row>
     <row r="22">
@@ -10134,7 +10134,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="C22" t="n">
         <v>1</v>
@@ -10164,19 +10164,19 @@
         <v>1</v>
       </c>
       <c r="L22" t="n">
-        <v>0.9630069999999999</v>
+        <v>0.984867</v>
       </c>
       <c r="M22" t="n">
         <v>1</v>
       </c>
       <c r="N22" t="n">
-        <v>0</v>
+        <v>0.008</v>
       </c>
       <c r="O22" t="n">
-        <v>0</v>
+        <v>0.002197</v>
       </c>
       <c r="P22" t="n">
-        <v>0.036993</v>
+        <v>0.028695</v>
       </c>
       <c r="Q22" t="n">
         <v>13</v>
@@ -10185,7 +10185,7 @@
         <v>1</v>
       </c>
       <c r="S22" t="n">
-        <v>0.006316</v>
+        <v>0.009006</v>
       </c>
     </row>
     <row r="23">
@@ -10195,7 +10195,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="C23" t="n">
         <v>1</v>
@@ -10225,19 +10225,19 @@
         <v>1</v>
       </c>
       <c r="L23" t="n">
-        <v>0.9630069999999999</v>
+        <v>0.984867</v>
       </c>
       <c r="M23" t="n">
         <v>1</v>
       </c>
       <c r="N23" t="n">
-        <v>0</v>
+        <v>0.008</v>
       </c>
       <c r="O23" t="n">
-        <v>0</v>
+        <v>0.002197</v>
       </c>
       <c r="P23" t="n">
-        <v>0.036993</v>
+        <v>0.028695</v>
       </c>
       <c r="Q23" t="n">
         <v>13</v>
@@ -10246,7 +10246,7 @@
         <v>1</v>
       </c>
       <c r="S23" t="n">
-        <v>0.004211</v>
+        <v>0.008704</v>
       </c>
     </row>
     <row r="24">
@@ -10256,7 +10256,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="C24" t="n">
         <v>1</v>
@@ -10286,19 +10286,19 @@
         <v>1</v>
       </c>
       <c r="L24" t="n">
-        <v>0.9630069999999999</v>
+        <v>0.984867</v>
       </c>
       <c r="M24" t="n">
         <v>1</v>
       </c>
       <c r="N24" t="n">
-        <v>0.01</v>
+        <v>0.012</v>
       </c>
       <c r="O24" t="n">
-        <v>0.001767</v>
+        <v>0.004089</v>
       </c>
       <c r="P24" t="n">
-        <v>0.054486</v>
+        <v>0.034681</v>
       </c>
       <c r="Q24" t="n">
         <v>13</v>
@@ -10307,7 +10307,7 @@
         <v>1</v>
       </c>
       <c r="S24" t="n">
-        <v>0.014211</v>
+        <v>0.012704</v>
       </c>
     </row>
     <row r="25">
@@ -10317,7 +10317,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="C25" t="n">
         <v>1</v>
@@ -10347,19 +10347,19 @@
         <v>1</v>
       </c>
       <c r="L25" t="n">
-        <v>0.9630069999999999</v>
+        <v>0.984867</v>
       </c>
       <c r="M25" t="n">
         <v>1</v>
       </c>
       <c r="N25" t="n">
-        <v>0.01</v>
+        <v>0.016</v>
       </c>
       <c r="O25" t="n">
-        <v>0.001767</v>
+        <v>0.006239</v>
       </c>
       <c r="P25" t="n">
-        <v>0.054486</v>
+        <v>0.04041</v>
       </c>
       <c r="Q25" t="n">
         <v>13</v>
@@ -10368,7 +10368,7 @@
         <v>1</v>
       </c>
       <c r="S25" t="n">
-        <v>0.018421</v>
+        <v>0.016906</v>
       </c>
     </row>
     <row r="26">
@@ -10378,22 +10378,22 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="C26" t="n">
-        <v>0.998125</v>
+        <v>0.9985000000000001</v>
       </c>
       <c r="D26" t="n">
-        <v>0.010715</v>
+        <v>0.009585</v>
       </c>
       <c r="E26" t="n">
-        <v>0.001072</v>
+        <v>0.000606</v>
       </c>
       <c r="F26" t="n">
-        <v>0.996025</v>
+        <v>0.997312</v>
       </c>
       <c r="G26" t="n">
-        <v>1.000225</v>
+        <v>0.999688</v>
       </c>
       <c r="H26" t="n">
         <v>1</v>
@@ -10408,19 +10408,19 @@
         <v>1</v>
       </c>
       <c r="L26" t="n">
-        <v>0.9630069999999999</v>
+        <v>0.984867</v>
       </c>
       <c r="M26" t="n">
         <v>1</v>
       </c>
       <c r="N26" t="n">
-        <v>0.02</v>
+        <v>0.012</v>
       </c>
       <c r="O26" t="n">
-        <v>0.005502</v>
+        <v>0.004089</v>
       </c>
       <c r="P26" t="n">
-        <v>0.070012</v>
+        <v>0.034681</v>
       </c>
       <c r="Q26" t="n">
         <v>13</v>
@@ -10429,7 +10429,7 @@
         <v>1</v>
       </c>
       <c r="S26" t="n">
-        <v>0.026316</v>
+        <v>0.012704</v>
       </c>
     </row>
     <row r="27">
@@ -10439,40 +10439,40 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="C27" t="n">
-        <v>0.54875</v>
+        <v>0.523</v>
       </c>
       <c r="D27" t="n">
-        <v>0.133422</v>
+        <v>0.126009</v>
       </c>
       <c r="E27" t="n">
-        <v>0.013342</v>
+        <v>0.00797</v>
       </c>
       <c r="F27" t="n">
-        <v>0.5226</v>
+        <v>0.5073800000000001</v>
       </c>
       <c r="G27" t="n">
-        <v>0.5749</v>
+        <v>0.53862</v>
       </c>
       <c r="H27" t="n">
-        <v>0.6007</v>
+        <v>0.543632</v>
       </c>
       <c r="I27" t="n">
-        <v>0.522331</v>
+        <v>0.488739</v>
       </c>
       <c r="J27" t="n">
-        <v>0.675755</v>
+        <v>0.594282</v>
       </c>
       <c r="K27" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="L27" t="n">
-        <v>0.010255</v>
+        <v>0.008572</v>
       </c>
       <c r="M27" t="n">
-        <v>0.084519</v>
+        <v>0.045956</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
@@ -10481,16 +10481,16 @@
         <v>0</v>
       </c>
       <c r="P27" t="n">
-        <v>0.036993</v>
+        <v>0.015133</v>
       </c>
       <c r="Q27" t="n">
         <v>13</v>
       </c>
       <c r="R27" t="n">
-        <v>0.046842</v>
+        <v>0.021208</v>
       </c>
       <c r="S27" t="n">
-        <v>0.006316</v>
+        <v>0.000503</v>
       </c>
     </row>
     <row r="29">
@@ -12039,10 +12039,10 @@
         <v>13</v>
       </c>
       <c r="D3" t="n">
-        <v>2000</v>
+        <v>6000</v>
       </c>
       <c r="E3" t="n">
-        <v>0.006</v>
+        <v>0.009332999999999999</v>
       </c>
       <c r="F3" t="n">
         <v>0.01</v>
@@ -12051,7 +12051,7 @@
         <v>13</v>
       </c>
       <c r="H3" t="n">
-        <v>0.210526</v>
+        <v>0.025157</v>
       </c>
     </row>
     <row r="4">
@@ -15892,7 +15892,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="E42" t="n">
         <v>1</v>
@@ -15922,19 +15922,19 @@
         <v>1</v>
       </c>
       <c r="N42" t="n">
-        <v>0.928652</v>
+        <v>0.97503</v>
       </c>
       <c r="O42" t="n">
         <v>1</v>
       </c>
       <c r="P42" t="n">
-        <v>0</v>
+        <v>0.006667</v>
       </c>
       <c r="Q42" t="n">
-        <v>0</v>
+        <v>0.001178</v>
       </c>
       <c r="R42" t="n">
-        <v>0.07134799999999999</v>
+        <v>0.036793</v>
       </c>
       <c r="S42" t="n">
         <v>13</v>
@@ -15943,7 +15943,7 @@
         <v>1</v>
       </c>
       <c r="U42" t="n">
-        <v>0</v>
+        <v>0.006834</v>
       </c>
     </row>
     <row r="43">
@@ -15963,7 +15963,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="E43" t="n">
         <v>1</v>
@@ -15993,19 +15993,19 @@
         <v>1</v>
       </c>
       <c r="N43" t="n">
-        <v>0.928652</v>
+        <v>0.97503</v>
       </c>
       <c r="O43" t="n">
         <v>1</v>
       </c>
       <c r="P43" t="n">
-        <v>0</v>
+        <v>0.013333</v>
       </c>
       <c r="Q43" t="n">
-        <v>0</v>
+        <v>0.003664</v>
       </c>
       <c r="R43" t="n">
-        <v>0.07134799999999999</v>
+        <v>0.047307</v>
       </c>
       <c r="S43" t="n">
         <v>13</v>
@@ -16014,7 +16014,7 @@
         <v>1</v>
       </c>
       <c r="U43" t="n">
-        <v>0</v>
+        <v>0.013501</v>
       </c>
     </row>
     <row r="44">
@@ -16034,58 +16034,58 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="E44" t="n">
         <v>0.8125</v>
       </c>
       <c r="F44" t="n">
-        <v>0.123718</v>
+        <v>0.123311</v>
       </c>
       <c r="G44" t="n">
-        <v>0.017496</v>
+        <v>0.010068</v>
       </c>
       <c r="H44" t="n">
-        <v>0.778208</v>
+        <v>0.792767</v>
       </c>
       <c r="I44" t="n">
-        <v>0.846792</v>
+        <v>0.832233</v>
       </c>
       <c r="J44" t="n">
-        <v>0.9698</v>
+        <v>0.945444</v>
       </c>
       <c r="K44" t="n">
-        <v>0.935995</v>
+        <v>0.918303</v>
       </c>
       <c r="L44" t="n">
-        <v>0.9936</v>
+        <v>0.968297</v>
       </c>
       <c r="M44" t="n">
-        <v>0.62</v>
+        <v>0.66</v>
       </c>
       <c r="N44" t="n">
-        <v>0.481504</v>
+        <v>0.581043</v>
       </c>
       <c r="O44" t="n">
-        <v>0.741372</v>
+        <v>0.730967</v>
       </c>
       <c r="P44" t="n">
-        <v>0.02</v>
+        <v>0.026667</v>
       </c>
       <c r="Q44" t="n">
-        <v>0.003539</v>
+        <v>0.010418</v>
       </c>
       <c r="R44" t="n">
-        <v>0.104954</v>
+        <v>0.066554</v>
       </c>
       <c r="S44" t="n">
         <v>13</v>
       </c>
       <c r="T44" t="n">
-        <v>0.653684</v>
+        <v>0.663019</v>
       </c>
       <c r="U44" t="n">
-        <v>0.024211</v>
+        <v>0.028176</v>
       </c>
     </row>
     <row r="45">
@@ -16105,7 +16105,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="E45" t="n">
         <v>1</v>
@@ -16135,19 +16135,19 @@
         <v>1</v>
       </c>
       <c r="N45" t="n">
-        <v>0.928652</v>
+        <v>0.97503</v>
       </c>
       <c r="O45" t="n">
         <v>1</v>
       </c>
       <c r="P45" t="n">
-        <v>0</v>
+        <v>0.006667</v>
       </c>
       <c r="Q45" t="n">
-        <v>0</v>
+        <v>0.001178</v>
       </c>
       <c r="R45" t="n">
-        <v>0.07134799999999999</v>
+        <v>0.036793</v>
       </c>
       <c r="S45" t="n">
         <v>13</v>
@@ -16156,7 +16156,7 @@
         <v>1</v>
       </c>
       <c r="U45" t="n">
-        <v>0</v>
+        <v>0.00717</v>
       </c>
     </row>
     <row r="46">
@@ -16176,7 +16176,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="E46" t="n">
         <v>1</v>
@@ -16206,19 +16206,19 @@
         <v>1</v>
       </c>
       <c r="N46" t="n">
-        <v>0.928652</v>
+        <v>0.97503</v>
       </c>
       <c r="O46" t="n">
         <v>1</v>
       </c>
       <c r="P46" t="n">
-        <v>0</v>
+        <v>0.006667</v>
       </c>
       <c r="Q46" t="n">
-        <v>0</v>
+        <v>0.001178</v>
       </c>
       <c r="R46" t="n">
-        <v>0.07134799999999999</v>
+        <v>0.036793</v>
       </c>
       <c r="S46" t="n">
         <v>13</v>
@@ -16227,7 +16227,7 @@
         <v>1</v>
       </c>
       <c r="U46" t="n">
-        <v>0</v>
+        <v>0.007338</v>
       </c>
     </row>
     <row r="47">
@@ -16247,7 +16247,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="E47" t="n">
         <v>1</v>
@@ -16277,19 +16277,19 @@
         <v>1</v>
       </c>
       <c r="N47" t="n">
-        <v>0.928652</v>
+        <v>0.97503</v>
       </c>
       <c r="O47" t="n">
         <v>1</v>
       </c>
       <c r="P47" t="n">
-        <v>0</v>
+        <v>0.013333</v>
       </c>
       <c r="Q47" t="n">
-        <v>0</v>
+        <v>0.003664</v>
       </c>
       <c r="R47" t="n">
-        <v>0.07134799999999999</v>
+        <v>0.047307</v>
       </c>
       <c r="S47" t="n">
         <v>13</v>
@@ -16298,7 +16298,7 @@
         <v>1</v>
       </c>
       <c r="U47" t="n">
-        <v>0</v>
+        <v>0.013501</v>
       </c>
     </row>
     <row r="48">
@@ -16318,7 +16318,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="E48" t="n">
         <v>1</v>
@@ -16348,19 +16348,19 @@
         <v>1</v>
       </c>
       <c r="N48" t="n">
-        <v>0.928652</v>
+        <v>0.97503</v>
       </c>
       <c r="O48" t="n">
         <v>1</v>
       </c>
       <c r="P48" t="n">
-        <v>0</v>
+        <v>0.006667</v>
       </c>
       <c r="Q48" t="n">
-        <v>0</v>
+        <v>0.001178</v>
       </c>
       <c r="R48" t="n">
-        <v>0.07134799999999999</v>
+        <v>0.036793</v>
       </c>
       <c r="S48" t="n">
         <v>13</v>
@@ -16369,7 +16369,7 @@
         <v>1</v>
       </c>
       <c r="U48" t="n">
-        <v>0</v>
+        <v>0.006834</v>
       </c>
     </row>
     <row r="49">
@@ -16389,7 +16389,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="E49" t="n">
         <v>1</v>
@@ -16419,19 +16419,19 @@
         <v>1</v>
       </c>
       <c r="N49" t="n">
-        <v>0.928652</v>
+        <v>0.97503</v>
       </c>
       <c r="O49" t="n">
         <v>1</v>
       </c>
       <c r="P49" t="n">
-        <v>0</v>
+        <v>0.013333</v>
       </c>
       <c r="Q49" t="n">
-        <v>0</v>
+        <v>0.003664</v>
       </c>
       <c r="R49" t="n">
-        <v>0.07134799999999999</v>
+        <v>0.047307</v>
       </c>
       <c r="S49" t="n">
         <v>13</v>
@@ -16440,7 +16440,7 @@
         <v>1</v>
       </c>
       <c r="U49" t="n">
-        <v>0</v>
+        <v>0.014004</v>
       </c>
     </row>
     <row r="50">
@@ -16460,58 +16460,58 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="E50" t="n">
-        <v>0.99125</v>
+        <v>0.99625</v>
       </c>
       <c r="F50" t="n">
-        <v>0.061872</v>
+        <v>0.036371</v>
       </c>
       <c r="G50" t="n">
-        <v>0.008750000000000001</v>
+        <v>0.00297</v>
       </c>
       <c r="H50" t="n">
-        <v>0.9741</v>
+        <v>0.990429</v>
       </c>
       <c r="I50" t="n">
-        <v>1.0084</v>
+        <v>1.002071</v>
       </c>
       <c r="J50" t="n">
-        <v>0.9946</v>
+        <v>0.997844</v>
       </c>
       <c r="K50" t="n">
-        <v>0.982</v>
+        <v>0.992667</v>
       </c>
       <c r="L50" t="n">
         <v>1</v>
       </c>
       <c r="M50" t="n">
-        <v>0.98</v>
+        <v>0.993333</v>
       </c>
       <c r="N50" t="n">
-        <v>0.895046</v>
+        <v>0.963207</v>
       </c>
       <c r="O50" t="n">
-        <v>0.996461</v>
+        <v>0.998822</v>
       </c>
       <c r="P50" t="n">
-        <v>0</v>
+        <v>0.013333</v>
       </c>
       <c r="Q50" t="n">
-        <v>0</v>
+        <v>0.003664</v>
       </c>
       <c r="R50" t="n">
-        <v>0.07134799999999999</v>
+        <v>0.047307</v>
       </c>
       <c r="S50" t="n">
         <v>13</v>
       </c>
       <c r="T50" t="n">
-        <v>0.98</v>
+        <v>0.993333</v>
       </c>
       <c r="U50" t="n">
-        <v>0.008421</v>
+        <v>0.014004</v>
       </c>
     </row>
     <row r="51">
@@ -16531,58 +16531,58 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="E51" t="n">
-        <v>0.54875</v>
+        <v>0.5325</v>
       </c>
       <c r="F51" t="n">
-        <v>0.128949</v>
+        <v>0.118479</v>
       </c>
       <c r="G51" t="n">
-        <v>0.018236</v>
+        <v>0.009674</v>
       </c>
       <c r="H51" t="n">
-        <v>0.513008</v>
+        <v>0.51354</v>
       </c>
       <c r="I51" t="n">
-        <v>0.584492</v>
+        <v>0.55146</v>
       </c>
       <c r="J51" t="n">
-        <v>0.6112</v>
+        <v>0.579956</v>
       </c>
       <c r="K51" t="n">
-        <v>0.498575</v>
+        <v>0.513798</v>
       </c>
       <c r="L51" t="n">
-        <v>0.72201</v>
+        <v>0.6444260000000001</v>
       </c>
       <c r="M51" t="n">
-        <v>0.02</v>
+        <v>0.006667</v>
       </c>
       <c r="N51" t="n">
-        <v>0.003539</v>
+        <v>0.001178</v>
       </c>
       <c r="O51" t="n">
-        <v>0.104954</v>
+        <v>0.036793</v>
       </c>
       <c r="P51" t="n">
-        <v>0.02</v>
+        <v>0.013333</v>
       </c>
       <c r="Q51" t="n">
-        <v>0.003539</v>
+        <v>0.003664</v>
       </c>
       <c r="R51" t="n">
-        <v>0.104954</v>
+        <v>0.047307</v>
       </c>
       <c r="S51" t="n">
         <v>13</v>
       </c>
       <c r="T51" t="n">
-        <v>0.045263</v>
+        <v>0.008512</v>
       </c>
       <c r="U51" t="n">
-        <v>0.02</v>
+        <v>0.014172</v>
       </c>
     </row>
     <row r="52">
@@ -16602,7 +16602,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="E52" t="n">
         <v>1</v>
@@ -16632,19 +16632,19 @@
         <v>1</v>
       </c>
       <c r="N52" t="n">
-        <v>0.928652</v>
+        <v>0.981155</v>
       </c>
       <c r="O52" t="n">
         <v>1</v>
       </c>
       <c r="P52" t="n">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="Q52" t="n">
-        <v>0</v>
+        <v>0.000883</v>
       </c>
       <c r="R52" t="n">
-        <v>0.07134799999999999</v>
+        <v>0.027774</v>
       </c>
       <c r="S52" t="n">
         <v>13</v>
@@ -16653,7 +16653,7 @@
         <v>1</v>
       </c>
       <c r="U52" t="n">
-        <v>0.004211</v>
+        <v>0.005629</v>
       </c>
     </row>
     <row r="53">
@@ -16673,7 +16673,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="E53" t="n">
         <v>1</v>
@@ -16703,19 +16703,19 @@
         <v>1</v>
       </c>
       <c r="N53" t="n">
-        <v>0.928652</v>
+        <v>0.981155</v>
       </c>
       <c r="O53" t="n">
         <v>1</v>
       </c>
       <c r="P53" t="n">
-        <v>0.02</v>
+        <v>0.015</v>
       </c>
       <c r="Q53" t="n">
-        <v>0.003539</v>
+        <v>0.005114</v>
       </c>
       <c r="R53" t="n">
-        <v>0.104954</v>
+        <v>0.043166</v>
       </c>
       <c r="S53" t="n">
         <v>13</v>
@@ -16724,7 +16724,7 @@
         <v>1</v>
       </c>
       <c r="U53" t="n">
-        <v>0.02</v>
+        <v>0.015252</v>
       </c>
     </row>
     <row r="54">
@@ -16744,58 +16744,58 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="E54" t="n">
-        <v>0.8225</v>
+        <v>0.815625</v>
       </c>
       <c r="F54" t="n">
-        <v>0.093097</v>
+        <v>0.102717</v>
       </c>
       <c r="G54" t="n">
-        <v>0.013166</v>
+        <v>0.007263</v>
       </c>
       <c r="H54" t="n">
-        <v>0.796695</v>
+        <v>0.801389</v>
       </c>
       <c r="I54" t="n">
-        <v>0.848305</v>
+        <v>0.829861</v>
       </c>
       <c r="J54" t="n">
-        <v>0.9893999999999999</v>
+        <v>0.9779870000000001</v>
       </c>
       <c r="K54" t="n">
-        <v>0.9746</v>
+        <v>0.9665820000000001</v>
       </c>
       <c r="L54" t="n">
-        <v>0.9986</v>
+        <v>0.987726</v>
       </c>
       <c r="M54" t="n">
-        <v>0.66</v>
+        <v>0.655</v>
       </c>
       <c r="N54" t="n">
-        <v>0.5215379999999999</v>
+        <v>0.5867560000000001</v>
       </c>
       <c r="O54" t="n">
-        <v>0.775631</v>
+        <v>0.717402</v>
       </c>
       <c r="P54" t="n">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="Q54" t="n">
-        <v>0</v>
+        <v>0.000883</v>
       </c>
       <c r="R54" t="n">
-        <v>0.07134799999999999</v>
+        <v>0.027774</v>
       </c>
       <c r="S54" t="n">
         <v>13</v>
       </c>
       <c r="T54" t="n">
-        <v>0.7063160000000001</v>
+        <v>0.659403</v>
       </c>
       <c r="U54" t="n">
-        <v>0.004211</v>
+        <v>0.005503</v>
       </c>
     </row>
     <row r="55">
@@ -16815,7 +16815,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="E55" t="n">
         <v>1</v>
@@ -16845,19 +16845,19 @@
         <v>1</v>
       </c>
       <c r="N55" t="n">
-        <v>0.928652</v>
+        <v>0.981155</v>
       </c>
       <c r="O55" t="n">
         <v>1</v>
       </c>
       <c r="P55" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="Q55" t="n">
-        <v>0</v>
+        <v>0.002747</v>
       </c>
       <c r="R55" t="n">
-        <v>0.07134799999999999</v>
+        <v>0.035722</v>
       </c>
       <c r="S55" t="n">
         <v>13</v>
@@ -16866,7 +16866,7 @@
         <v>1</v>
       </c>
       <c r="U55" t="n">
-        <v>0.012632</v>
+        <v>0.010755</v>
       </c>
     </row>
     <row r="56">
@@ -16886,7 +16886,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="E56" t="n">
         <v>1</v>
@@ -16916,19 +16916,19 @@
         <v>1</v>
       </c>
       <c r="N56" t="n">
-        <v>0.928652</v>
+        <v>0.981155</v>
       </c>
       <c r="O56" t="n">
         <v>1</v>
       </c>
       <c r="P56" t="n">
-        <v>0.02</v>
+        <v>0.015</v>
       </c>
       <c r="Q56" t="n">
-        <v>0.003539</v>
+        <v>0.005114</v>
       </c>
       <c r="R56" t="n">
-        <v>0.104954</v>
+        <v>0.043166</v>
       </c>
       <c r="S56" t="n">
         <v>13</v>
@@ -16937,7 +16937,7 @@
         <v>1</v>
       </c>
       <c r="U56" t="n">
-        <v>0.024211</v>
+        <v>0.015503</v>
       </c>
     </row>
     <row r="57">
@@ -16957,7 +16957,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="E57" t="n">
         <v>1</v>
@@ -16987,7 +16987,7 @@
         <v>1</v>
       </c>
       <c r="N57" t="n">
-        <v>0.928652</v>
+        <v>0.981155</v>
       </c>
       <c r="O57" t="n">
         <v>1</v>
@@ -16999,7 +16999,7 @@
         <v>0</v>
       </c>
       <c r="R57" t="n">
-        <v>0.07134799999999999</v>
+        <v>0.018845</v>
       </c>
       <c r="S57" t="n">
         <v>13</v>
@@ -17008,7 +17008,7 @@
         <v>1</v>
       </c>
       <c r="U57" t="n">
-        <v>0</v>
+        <v>0.000629</v>
       </c>
     </row>
     <row r="58">
@@ -17028,7 +17028,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="E58" t="n">
         <v>1</v>
@@ -17058,19 +17058,19 @@
         <v>1</v>
       </c>
       <c r="N58" t="n">
-        <v>0.928652</v>
+        <v>0.981155</v>
       </c>
       <c r="O58" t="n">
         <v>1</v>
       </c>
       <c r="P58" t="n">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="Q58" t="n">
-        <v>0</v>
+        <v>0.000883</v>
       </c>
       <c r="R58" t="n">
-        <v>0.07134799999999999</v>
+        <v>0.027774</v>
       </c>
       <c r="S58" t="n">
         <v>13</v>
@@ -17079,7 +17079,7 @@
         <v>1</v>
       </c>
       <c r="U58" t="n">
-        <v>0.004211</v>
+        <v>0.005629</v>
       </c>
     </row>
     <row r="59">
@@ -17099,7 +17099,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="E59" t="n">
         <v>1</v>
@@ -17129,19 +17129,19 @@
         <v>1</v>
       </c>
       <c r="N59" t="n">
-        <v>0.928652</v>
+        <v>0.981155</v>
       </c>
       <c r="O59" t="n">
         <v>1</v>
       </c>
       <c r="P59" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="Q59" t="n">
-        <v>0.003539</v>
+        <v>0.002747</v>
       </c>
       <c r="R59" t="n">
-        <v>0.104954</v>
+        <v>0.035722</v>
       </c>
       <c r="S59" t="n">
         <v>13</v>
@@ -17150,7 +17150,7 @@
         <v>1</v>
       </c>
       <c r="U59" t="n">
-        <v>0.02</v>
+        <v>0.010755</v>
       </c>
     </row>
     <row r="60">
@@ -17170,7 +17170,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="E60" t="n">
         <v>1</v>
@@ -17200,19 +17200,19 @@
         <v>1</v>
       </c>
       <c r="N60" t="n">
-        <v>0.928652</v>
+        <v>0.981155</v>
       </c>
       <c r="O60" t="n">
         <v>1</v>
       </c>
       <c r="P60" t="n">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="Q60" t="n">
-        <v>0</v>
+        <v>0.000883</v>
       </c>
       <c r="R60" t="n">
-        <v>0.07134799999999999</v>
+        <v>0.027774</v>
       </c>
       <c r="S60" t="n">
         <v>13</v>
@@ -17221,7 +17221,7 @@
         <v>1</v>
       </c>
       <c r="U60" t="n">
-        <v>0.012632</v>
+        <v>0.006635</v>
       </c>
     </row>
     <row r="61">
@@ -17241,58 +17241,58 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="E61" t="n">
-        <v>0.5675</v>
+        <v>0.537188</v>
       </c>
       <c r="F61" t="n">
-        <v>0.133535</v>
+        <v>0.129033</v>
       </c>
       <c r="G61" t="n">
-        <v>0.018885</v>
+        <v>0.009124</v>
       </c>
       <c r="H61" t="n">
-        <v>0.530487</v>
+        <v>0.519305</v>
       </c>
       <c r="I61" t="n">
-        <v>0.604513</v>
+        <v>0.55507</v>
       </c>
       <c r="J61" t="n">
-        <v>0.6258</v>
+        <v>0.56525</v>
       </c>
       <c r="K61" t="n">
-        <v>0.519755</v>
+        <v>0.51131</v>
       </c>
       <c r="L61" t="n">
-        <v>0.726805</v>
+        <v>0.620413</v>
       </c>
       <c r="M61" t="n">
-        <v>0.06</v>
+        <v>0.03</v>
       </c>
       <c r="N61" t="n">
-        <v>0.020615</v>
+        <v>0.01382</v>
       </c>
       <c r="O61" t="n">
-        <v>0.162171</v>
+        <v>0.06389400000000001</v>
       </c>
       <c r="P61" t="n">
-        <v>0.02</v>
+        <v>0.005</v>
       </c>
       <c r="Q61" t="n">
-        <v>0.003539</v>
+        <v>0.000883</v>
       </c>
       <c r="R61" t="n">
-        <v>0.104954</v>
+        <v>0.027774</v>
       </c>
       <c r="S61" t="n">
         <v>13</v>
       </c>
       <c r="T61" t="n">
-        <v>0.072632</v>
+        <v>0.030881</v>
       </c>
       <c r="U61" t="n">
-        <v>0.024211</v>
+        <v>0.006006</v>
       </c>
     </row>
     <row r="62">
@@ -17312,7 +17312,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="E62" t="n">
         <v>1</v>
@@ -17342,19 +17342,19 @@
         <v>1</v>
       </c>
       <c r="N62" t="n">
-        <v>0.9630069999999999</v>
+        <v>0.984867</v>
       </c>
       <c r="O62" t="n">
         <v>1</v>
       </c>
       <c r="P62" t="n">
-        <v>0.01</v>
+        <v>0.012</v>
       </c>
       <c r="Q62" t="n">
-        <v>0.001767</v>
+        <v>0.004089</v>
       </c>
       <c r="R62" t="n">
-        <v>0.054486</v>
+        <v>0.034681</v>
       </c>
       <c r="S62" t="n">
         <v>13</v>
@@ -17363,7 +17363,7 @@
         <v>1</v>
       </c>
       <c r="U62" t="n">
-        <v>0.014211</v>
+        <v>0.012704</v>
       </c>
     </row>
     <row r="63">
@@ -17383,7 +17383,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="E63" t="n">
         <v>1</v>
@@ -17413,19 +17413,19 @@
         <v>1</v>
       </c>
       <c r="N63" t="n">
-        <v>0.9630069999999999</v>
+        <v>0.984867</v>
       </c>
       <c r="O63" t="n">
         <v>1</v>
       </c>
       <c r="P63" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
       <c r="Q63" t="n">
-        <v>0</v>
+        <v>0.000706</v>
       </c>
       <c r="R63" t="n">
-        <v>0.036993</v>
+        <v>0.022306</v>
       </c>
       <c r="S63" t="n">
         <v>13</v>
@@ -17434,7 +17434,7 @@
         <v>1</v>
       </c>
       <c r="U63" t="n">
-        <v>0.002105</v>
+        <v>0.004704</v>
       </c>
     </row>
     <row r="64">
@@ -17454,58 +17454,58 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="E64" t="n">
-        <v>0.7625</v>
+        <v>0.757</v>
       </c>
       <c r="F64" t="n">
-        <v>0.130256</v>
+        <v>0.131654</v>
       </c>
       <c r="G64" t="n">
-        <v>0.013026</v>
+        <v>0.008326999999999999</v>
       </c>
       <c r="H64" t="n">
-        <v>0.73697</v>
+        <v>0.74068</v>
       </c>
       <c r="I64" t="n">
-        <v>0.78803</v>
+        <v>0.77332</v>
       </c>
       <c r="J64" t="n">
-        <v>0.94795</v>
+        <v>0.9302240000000001</v>
       </c>
       <c r="K64" t="n">
-        <v>0.92055</v>
+        <v>0.91047</v>
       </c>
       <c r="L64" t="n">
-        <v>0.9717</v>
+        <v>0.948041</v>
       </c>
       <c r="M64" t="n">
-        <v>0.44</v>
+        <v>0.456</v>
       </c>
       <c r="N64" t="n">
-        <v>0.34672</v>
+        <v>0.395392</v>
       </c>
       <c r="O64" t="n">
-        <v>0.5377189999999999</v>
+        <v>0.51794</v>
       </c>
       <c r="P64" t="n">
-        <v>0</v>
+        <v>0.008</v>
       </c>
       <c r="Q64" t="n">
-        <v>0</v>
+        <v>0.002197</v>
       </c>
       <c r="R64" t="n">
-        <v>0.036993</v>
+        <v>0.028695</v>
       </c>
       <c r="S64" t="n">
         <v>13</v>
       </c>
       <c r="T64" t="n">
-        <v>0.475789</v>
+        <v>0.460226</v>
       </c>
       <c r="U64" t="n">
-        <v>0.004211</v>
+        <v>0.008503</v>
       </c>
     </row>
     <row r="65">
@@ -17525,7 +17525,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="E65" t="n">
         <v>1</v>
@@ -17555,19 +17555,19 @@
         <v>1</v>
       </c>
       <c r="N65" t="n">
-        <v>0.9630069999999999</v>
+        <v>0.984867</v>
       </c>
       <c r="O65" t="n">
         <v>1</v>
       </c>
       <c r="P65" t="n">
-        <v>0.01</v>
+        <v>0.012</v>
       </c>
       <c r="Q65" t="n">
-        <v>0.001767</v>
+        <v>0.004089</v>
       </c>
       <c r="R65" t="n">
-        <v>0.054486</v>
+        <v>0.034681</v>
       </c>
       <c r="S65" t="n">
         <v>13</v>
@@ -17576,7 +17576,7 @@
         <v>1</v>
       </c>
       <c r="U65" t="n">
-        <v>0.014211</v>
+        <v>0.012403</v>
       </c>
     </row>
     <row r="66">
@@ -17596,7 +17596,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="E66" t="n">
         <v>1</v>
@@ -17626,19 +17626,19 @@
         <v>1</v>
       </c>
       <c r="N66" t="n">
-        <v>0.9630069999999999</v>
+        <v>0.984867</v>
       </c>
       <c r="O66" t="n">
         <v>1</v>
       </c>
       <c r="P66" t="n">
-        <v>0</v>
+        <v>0.008</v>
       </c>
       <c r="Q66" t="n">
-        <v>0</v>
+        <v>0.002197</v>
       </c>
       <c r="R66" t="n">
-        <v>0.036993</v>
+        <v>0.028695</v>
       </c>
       <c r="S66" t="n">
         <v>13</v>
@@ -17647,7 +17647,7 @@
         <v>1</v>
       </c>
       <c r="U66" t="n">
-        <v>0.006316</v>
+        <v>0.009006</v>
       </c>
     </row>
     <row r="67">
@@ -17667,7 +17667,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="E67" t="n">
         <v>1</v>
@@ -17697,19 +17697,19 @@
         <v>1</v>
       </c>
       <c r="N67" t="n">
-        <v>0.9630069999999999</v>
+        <v>0.984867</v>
       </c>
       <c r="O67" t="n">
         <v>1</v>
       </c>
       <c r="P67" t="n">
-        <v>0</v>
+        <v>0.008</v>
       </c>
       <c r="Q67" t="n">
-        <v>0</v>
+        <v>0.002197</v>
       </c>
       <c r="R67" t="n">
-        <v>0.036993</v>
+        <v>0.028695</v>
       </c>
       <c r="S67" t="n">
         <v>13</v>
@@ -17718,7 +17718,7 @@
         <v>1</v>
       </c>
       <c r="U67" t="n">
-        <v>0.004211</v>
+        <v>0.008704</v>
       </c>
     </row>
     <row r="68">
@@ -17738,7 +17738,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="E68" t="n">
         <v>1</v>
@@ -17768,19 +17768,19 @@
         <v>1</v>
       </c>
       <c r="N68" t="n">
-        <v>0.9630069999999999</v>
+        <v>0.984867</v>
       </c>
       <c r="O68" t="n">
         <v>1</v>
       </c>
       <c r="P68" t="n">
-        <v>0.01</v>
+        <v>0.012</v>
       </c>
       <c r="Q68" t="n">
-        <v>0.001767</v>
+        <v>0.004089</v>
       </c>
       <c r="R68" t="n">
-        <v>0.054486</v>
+        <v>0.034681</v>
       </c>
       <c r="S68" t="n">
         <v>13</v>
@@ -17789,7 +17789,7 @@
         <v>1</v>
       </c>
       <c r="U68" t="n">
-        <v>0.014211</v>
+        <v>0.012704</v>
       </c>
     </row>
     <row r="69">
@@ -17809,7 +17809,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="E69" t="n">
         <v>1</v>
@@ -17839,19 +17839,19 @@
         <v>1</v>
       </c>
       <c r="N69" t="n">
-        <v>0.9630069999999999</v>
+        <v>0.984867</v>
       </c>
       <c r="O69" t="n">
         <v>1</v>
       </c>
       <c r="P69" t="n">
-        <v>0.01</v>
+        <v>0.016</v>
       </c>
       <c r="Q69" t="n">
-        <v>0.001767</v>
+        <v>0.006239</v>
       </c>
       <c r="R69" t="n">
-        <v>0.054486</v>
+        <v>0.04041</v>
       </c>
       <c r="S69" t="n">
         <v>13</v>
@@ -17860,7 +17860,7 @@
         <v>1</v>
       </c>
       <c r="U69" t="n">
-        <v>0.018421</v>
+        <v>0.016906</v>
       </c>
     </row>
     <row r="70">
@@ -17880,22 +17880,22 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="E70" t="n">
-        <v>0.998125</v>
+        <v>0.9985000000000001</v>
       </c>
       <c r="F70" t="n">
-        <v>0.010715</v>
+        <v>0.009585</v>
       </c>
       <c r="G70" t="n">
-        <v>0.001072</v>
+        <v>0.000606</v>
       </c>
       <c r="H70" t="n">
-        <v>0.996025</v>
+        <v>0.997312</v>
       </c>
       <c r="I70" t="n">
-        <v>1.000225</v>
+        <v>0.999688</v>
       </c>
       <c r="J70" t="n">
         <v>1</v>
@@ -17910,19 +17910,19 @@
         <v>1</v>
       </c>
       <c r="N70" t="n">
-        <v>0.9630069999999999</v>
+        <v>0.984867</v>
       </c>
       <c r="O70" t="n">
         <v>1</v>
       </c>
       <c r="P70" t="n">
-        <v>0.02</v>
+        <v>0.012</v>
       </c>
       <c r="Q70" t="n">
-        <v>0.005502</v>
+        <v>0.004089</v>
       </c>
       <c r="R70" t="n">
-        <v>0.070012</v>
+        <v>0.034681</v>
       </c>
       <c r="S70" t="n">
         <v>13</v>
@@ -17931,7 +17931,7 @@
         <v>1</v>
       </c>
       <c r="U70" t="n">
-        <v>0.026316</v>
+        <v>0.012704</v>
       </c>
     </row>
     <row r="71">
@@ -17951,40 +17951,40 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="E71" t="n">
-        <v>0.54875</v>
+        <v>0.523</v>
       </c>
       <c r="F71" t="n">
-        <v>0.133422</v>
+        <v>0.126009</v>
       </c>
       <c r="G71" t="n">
-        <v>0.013342</v>
+        <v>0.00797</v>
       </c>
       <c r="H71" t="n">
-        <v>0.5226</v>
+        <v>0.5073800000000001</v>
       </c>
       <c r="I71" t="n">
-        <v>0.5749</v>
+        <v>0.53862</v>
       </c>
       <c r="J71" t="n">
-        <v>0.6007</v>
+        <v>0.543632</v>
       </c>
       <c r="K71" t="n">
-        <v>0.522331</v>
+        <v>0.488739</v>
       </c>
       <c r="L71" t="n">
-        <v>0.675755</v>
+        <v>0.594282</v>
       </c>
       <c r="M71" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="N71" t="n">
-        <v>0.010255</v>
+        <v>0.008572</v>
       </c>
       <c r="O71" t="n">
-        <v>0.084519</v>
+        <v>0.045956</v>
       </c>
       <c r="P71" t="n">
         <v>0</v>
@@ -17993,16 +17993,16 @@
         <v>0</v>
       </c>
       <c r="R71" t="n">
-        <v>0.036993</v>
+        <v>0.015133</v>
       </c>
       <c r="S71" t="n">
         <v>13</v>
       </c>
       <c r="T71" t="n">
-        <v>0.046842</v>
+        <v>0.021208</v>
       </c>
       <c r="U71" t="n">
-        <v>0.006316</v>
+        <v>0.000503</v>
       </c>
     </row>
     <row r="72">

</xml_diff>